<commit_message>
Updated so I can quickly fit a profile several times with slightly different models to conditions. I also added SI Units to the parameter names in my excel database so that it is easier to remember how they are input
</commit_message>
<xml_diff>
--- a/Diffusion Round Robin/Round_Robin_Olivine_Profile_Diffusion_Modeling_Parameters_DB.xlsx
+++ b/Diffusion Round Robin/Round_Robin_Olivine_Profile_Diffusion_Modeling_Parameters_DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henrytowbin/Projects/Olivine_Diffusion_FeMg/Diffusion Round Robin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD61114-F283-FB44-BD42-46F7DDF4AA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701F8738-EFEE-A947-890A-1E13BF696D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4460" yWindow="1100" windowWidth="30240" windowHeight="18960" xr2:uid="{4BF80DE2-54EF-754E-B733-C83BF6E05191}"/>
+    <workbookView xWindow="-1560" yWindow="1220" windowWidth="30240" windowHeight="18960" xr2:uid="{4BF80DE2-54EF-754E-B733-C83BF6E05191}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="102">
   <si>
     <t>Sample</t>
   </si>
@@ -277,75 +277,9 @@
     <t>big ol2 azwht01 15</t>
   </si>
   <si>
-    <t>0, 31</t>
-  </si>
-  <si>
-    <t>0.5, 23</t>
-  </si>
-  <si>
-    <t>0.5, 26</t>
-  </si>
-  <si>
-    <t>Phenocryst_S_ol2_prof_1</t>
-  </si>
-  <si>
-    <t>AZ18 WHT06_ol40_prof 2</t>
-  </si>
-  <si>
-    <t>Xenolith WHT01</t>
-  </si>
-  <si>
-    <t>Xenolith WHT06</t>
-  </si>
-  <si>
-    <t>Xenolith WHT01 Contact Overgrowth</t>
-  </si>
-  <si>
-    <t>AZ18 WHT06_ol43_prof 1</t>
-  </si>
-  <si>
-    <t>AZ18 WHT06_ol48_prof 1</t>
-  </si>
-  <si>
-    <t>AZ18_Scoria_Ol48</t>
-  </si>
-  <si>
-    <t>Xenocryst_ol6_prof_1</t>
-  </si>
-  <si>
-    <t>Xenocryst_ol23_prof_1</t>
-  </si>
-  <si>
-    <t>Xenocryst_ol6_prof_2</t>
-  </si>
-  <si>
-    <t>1,19.5</t>
-  </si>
-  <si>
-    <t>1,24.6</t>
-  </si>
-  <si>
-    <t>2,35</t>
-  </si>
-  <si>
-    <t>AZ18 WHT06_ol44_prof 1 filename is AZ18 WHT06_ol44_prof 1</t>
-  </si>
-  <si>
-    <t>Xenolith GCB1</t>
-  </si>
-  <si>
-    <t>Xenocryst</t>
-  </si>
-  <si>
     <t>Histogram_Color</t>
   </si>
   <si>
-    <t>10, 33</t>
-  </si>
-  <si>
-    <t>I think the dt and dx are larger here since this is a longer timescale phenocryst grain</t>
-  </si>
-  <si>
     <t>alpha</t>
   </si>
   <si>
@@ -355,9 +289,6 @@
     <t>gamma</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
     <t>KS20-527_2-transect</t>
   </si>
   <si>
@@ -376,9 +307,6 @@
     <t>Round Robin</t>
   </si>
   <si>
-    <t>fO2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Presure and fO2in Pascals </t>
   </si>
   <si>
@@ -392,6 +320,30 @@
   </si>
   <si>
     <t>0, 20</t>
+  </si>
+  <si>
+    <t>P isnt too useful for determining the step position. The derivative  of the smoothed data is more useful.</t>
+  </si>
+  <si>
+    <t>P spikes at 36.6µm but profiles don’t actually need to be fit.</t>
+  </si>
+  <si>
+    <t>max_model_time_days</t>
+  </si>
+  <si>
+    <t>dt_s</t>
+  </si>
+  <si>
+    <t>dx_um</t>
+  </si>
+  <si>
+    <t>T_C</t>
+  </si>
+  <si>
+    <t>P_Pa</t>
+  </si>
+  <si>
+    <t>fO2_Pa</t>
   </si>
 </sst>
 </file>
@@ -515,7 +467,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -523,7 +475,47 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -864,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D2757E0-7F0F-D849-AAD1-AAB451BA4D11}">
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Z48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.83203125" customWidth="1"/>
@@ -878,11 +870,11 @@
     <col min="17" max="17" width="16.6640625" customWidth="1"/>
     <col min="20" max="20" width="22.83203125" customWidth="1"/>
     <col min="21" max="21" width="21.5" customWidth="1"/>
-    <col min="23" max="23" width="21.33203125" customWidth="1"/>
-    <col min="24" max="24" width="36.1640625" style="7" customWidth="1"/>
+    <col min="24" max="24" width="21.33203125" customWidth="1"/>
+    <col min="25" max="25" width="36.1640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -899,13 +891,13 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="H1" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="I1" t="s">
         <v>7</v>
@@ -935,1631 +927,536 @@
         <v>72</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="X1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="Y1" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>14</v>
+      <c r="Z1" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
+        <v>88</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
+      <c r="F2" s="9">
+        <v>88</v>
+      </c>
+      <c r="G2" s="10">
+        <v>123</v>
+      </c>
+      <c r="H2" s="11">
+        <v>33</v>
+      </c>
       <c r="J2" t="s">
-        <v>105</v>
-      </c>
-      <c r="K2" s="1">
+        <v>68</v>
+      </c>
+      <c r="K2" s="13">
         <v>0</v>
       </c>
-      <c r="L2" s="1">
-        <v>48</v>
-      </c>
-      <c r="M2" t="s">
-        <v>80</v>
-      </c>
-      <c r="N2">
-        <v>5</v>
-      </c>
-      <c r="O2">
-        <v>91.5</v>
-      </c>
-      <c r="P2">
-        <v>90.25</v>
-      </c>
-      <c r="Q2" s="1">
+      <c r="L2" s="13">
+        <v>300</v>
+      </c>
+      <c r="M2" s="13">
+        <v>46</v>
+      </c>
+      <c r="O2" s="13">
+        <v>82</v>
+      </c>
+      <c r="P2" s="13">
+        <v>88.5</v>
+      </c>
+      <c r="R2">
+        <v>1200</v>
+      </c>
+      <c r="S2">
+        <f xml:space="preserve"> 100000 * 10^-7.86</f>
+        <v>1.3803842646028805E-3</v>
+      </c>
+      <c r="T2" s="8">
+        <f>42*10^6</f>
+        <v>42000000</v>
+      </c>
+      <c r="U2">
+        <v>600</v>
+      </c>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1"/>
+    </row>
+    <row r="3" spans="1:26" ht="136" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9">
+        <v>81</v>
+      </c>
+      <c r="G3" s="10">
+        <v>166</v>
+      </c>
+      <c r="H3" s="11">
+        <v>79</v>
+      </c>
+      <c r="J3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" s="13">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13">
+        <v>190</v>
+      </c>
+      <c r="M3">
+        <v>40</v>
+      </c>
+      <c r="O3">
+        <v>82.4</v>
+      </c>
+      <c r="P3">
+        <v>87.8</v>
+      </c>
+      <c r="R3">
+        <v>1200</v>
+      </c>
+      <c r="S3">
+        <f t="shared" ref="S3:S4" si="0" xml:space="preserve"> 100000 * 10^-7.86</f>
+        <v>1.3803842646028805E-3</v>
+      </c>
+      <c r="T3" s="8">
+        <f t="shared" ref="T3:T6" si="1">42*10^6</f>
+        <v>42000000</v>
+      </c>
+      <c r="U3">
+        <v>600</v>
+      </c>
+      <c r="V3" s="1">
+        <v>1</v>
+      </c>
+      <c r="W3" s="1"/>
+      <c r="Y3" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="204" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" s="9">
+        <v>119</v>
+      </c>
+      <c r="G4" s="10">
+        <v>110</v>
+      </c>
+      <c r="H4" s="11">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K4" s="13">
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <v>300</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="O4" s="2">
+        <v>82.6</v>
+      </c>
+      <c r="P4">
+        <v>85.9</v>
+      </c>
+      <c r="Q4">
+        <v>88.5</v>
+      </c>
+      <c r="R4">
+        <v>1200</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="0"/>
+        <v>1.3803842646028805E-3</v>
+      </c>
+      <c r="T4" s="8">
+        <f t="shared" si="1"/>
+        <v>42000000</v>
+      </c>
+      <c r="U4">
+        <v>600</v>
+      </c>
+      <c r="V4" s="1">
+        <v>1</v>
+      </c>
+      <c r="W4" s="1"/>
+      <c r="Y4" s="7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <v>60</v>
+      </c>
+      <c r="G5" s="10">
+        <v>30</v>
+      </c>
+      <c r="H5" s="11">
+        <v>90</v>
+      </c>
+      <c r="J5" t="s">
+        <v>68</v>
+      </c>
+      <c r="K5" s="13">
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <v>150</v>
+      </c>
+      <c r="M5" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S2" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T2" s="3">
-        <f>1000000000/2</f>
-        <v>500000000</v>
-      </c>
-      <c r="U2">
-        <v>60</v>
-      </c>
-      <c r="V2" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>97</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3">
+      <c r="O5">
+        <v>67</v>
+      </c>
+      <c r="P5">
+        <v>60.5</v>
+      </c>
+      <c r="Q5">
+        <v>74.5</v>
+      </c>
+      <c r="R5" s="12">
+        <v>1102</v>
+      </c>
+      <c r="S5">
+        <f xml:space="preserve"> 100000 * 10^-8.74</f>
+        <v>1.8197008586099805E-4</v>
+      </c>
+      <c r="T5" s="8">
+        <f t="shared" si="1"/>
+        <v>42000000</v>
+      </c>
+      <c r="U5">
+        <v>120</v>
+      </c>
+      <c r="V5" s="1">
+        <v>1</v>
+      </c>
+      <c r="W5" s="1"/>
+      <c r="Y5" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="34" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="9">
+        <v>89</v>
+      </c>
+      <c r="G6" s="10">
         <v>3</v>
       </c>
-      <c r="J3" t="s">
-        <v>105</v>
-      </c>
-      <c r="R3" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S3" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T3" s="3">
-        <f t="shared" ref="T3:T26" si="0">1000000000/2</f>
-        <v>500000000</v>
-      </c>
-      <c r="U3">
-        <v>60</v>
-      </c>
-      <c r="V3" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="J4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K4">
+      <c r="H6" s="11">
+        <v>88</v>
+      </c>
+      <c r="J6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" s="13">
         <v>0</v>
       </c>
-      <c r="L4">
-        <v>55</v>
-      </c>
-      <c r="M4" t="s">
-        <v>81</v>
-      </c>
-      <c r="N4">
-        <v>5</v>
-      </c>
-      <c r="O4">
-        <v>91.5</v>
-      </c>
-      <c r="P4">
-        <v>90.46</v>
-      </c>
-      <c r="Q4">
-        <v>93</v>
-      </c>
-      <c r="R4" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S4" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T4" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U4">
-        <v>60</v>
-      </c>
-      <c r="V4" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="J5" t="s">
-        <v>105</v>
-      </c>
-      <c r="R5" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S5" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T5" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U5">
-        <v>60</v>
-      </c>
-      <c r="V5" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" t="s">
-        <v>105</v>
-      </c>
-      <c r="R6" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S6" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T6" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
+      <c r="L6" s="13">
+        <v>160</v>
+      </c>
+      <c r="M6" s="13">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>73</v>
+      </c>
+      <c r="P6">
+        <v>62.6</v>
+      </c>
+      <c r="R6" s="12">
+        <v>1102</v>
+      </c>
+      <c r="S6">
+        <f xml:space="preserve"> 100000 * 10^-8.74</f>
+        <v>1.8197008586099805E-4</v>
+      </c>
+      <c r="T6" s="8">
+        <f t="shared" si="1"/>
+        <v>42000000</v>
       </c>
       <c r="U6">
-        <v>60</v>
+        <v>600</v>
       </c>
       <c r="V6" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7">
         <v>1</v>
       </c>
-      <c r="J7" t="s">
-        <v>105</v>
-      </c>
-      <c r="K7">
-        <v>2</v>
-      </c>
-      <c r="L7">
-        <v>48</v>
-      </c>
-      <c r="M7">
-        <v>18</v>
-      </c>
-      <c r="N7">
-        <v>4</v>
-      </c>
-      <c r="O7">
-        <v>92.93</v>
-      </c>
-      <c r="P7">
-        <v>90.5</v>
-      </c>
-      <c r="R7" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S7" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T7" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U7">
-        <v>60</v>
-      </c>
-      <c r="V7" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="J8" t="s">
-        <v>105</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>34</v>
-      </c>
-      <c r="M8">
-        <v>17</v>
-      </c>
-      <c r="N8">
-        <v>5</v>
-      </c>
-      <c r="O8">
-        <v>93.2</v>
-      </c>
-      <c r="P8">
-        <v>90.7</v>
-      </c>
-      <c r="R8" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S8" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T8" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U8">
-        <v>60</v>
-      </c>
-      <c r="V8" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="J9" t="s">
-        <v>105</v>
-      </c>
-      <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9">
-        <v>75</v>
-      </c>
-      <c r="M9" t="s">
-        <v>100</v>
-      </c>
-      <c r="N9">
-        <v>2</v>
-      </c>
-      <c r="O9">
-        <v>91.4</v>
-      </c>
-      <c r="P9">
-        <v>89.65</v>
-      </c>
-      <c r="Q9">
-        <v>93</v>
-      </c>
-      <c r="R9" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S9" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T9" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U9">
-        <v>60</v>
-      </c>
-      <c r="V9" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
-      <c r="J10" t="s">
-        <v>105</v>
-      </c>
-      <c r="R10" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S10" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T10" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U10">
-        <v>60</v>
-      </c>
-      <c r="V10" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="J11" t="s">
-        <v>105</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <v>47</v>
-      </c>
-      <c r="M11">
-        <v>15</v>
-      </c>
-      <c r="N11">
-        <v>5</v>
-      </c>
-      <c r="O11">
-        <v>91.5</v>
-      </c>
-      <c r="P11">
-        <v>89.68</v>
-      </c>
-      <c r="R11" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S11" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T11" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U11">
-        <v>60</v>
-      </c>
-      <c r="V11" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
-      <c r="J12" t="s">
-        <v>105</v>
-      </c>
-      <c r="R12" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S12" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T12" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U12">
-        <v>60</v>
-      </c>
-      <c r="V12" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" t="s">
-        <v>84</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="J13" t="s">
-        <v>105</v>
-      </c>
-      <c r="R13" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S13" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T13" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U13">
-        <v>60</v>
-      </c>
-      <c r="V13" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="J14" t="s">
-        <v>105</v>
-      </c>
-      <c r="K14">
-        <v>2.5</v>
-      </c>
-      <c r="L14">
-        <v>72</v>
-      </c>
-      <c r="M14">
-        <v>24</v>
-      </c>
-      <c r="N14">
-        <v>2</v>
-      </c>
-      <c r="O14">
-        <v>91.46</v>
-      </c>
-      <c r="P14">
-        <v>89.85</v>
-      </c>
-      <c r="R14" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S14" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T14" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U14">
-        <v>60</v>
-      </c>
-      <c r="V14" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="J15" t="s">
-        <v>105</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>150</v>
-      </c>
-      <c r="M15">
-        <v>22</v>
-      </c>
-      <c r="N15">
-        <v>2</v>
-      </c>
-      <c r="O15" s="2">
-        <v>82.7</v>
-      </c>
-      <c r="P15">
-        <v>89.49</v>
-      </c>
-      <c r="R15" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S15" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T15" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U15">
-        <v>60</v>
-      </c>
-      <c r="V15" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" t="s">
-        <v>86</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16">
-        <v>2</v>
-      </c>
-      <c r="J16" t="s">
-        <v>105</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>150</v>
-      </c>
-      <c r="M16">
-        <v>22</v>
-      </c>
-      <c r="N16">
-        <v>2</v>
-      </c>
-      <c r="O16" s="2">
-        <v>80</v>
-      </c>
-      <c r="P16">
-        <v>89.7</v>
-      </c>
-      <c r="R16" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S16" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T16" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U16">
-        <v>60</v>
-      </c>
-      <c r="V16" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="X16" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D17" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="J17" t="s">
-        <v>105</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>110</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>2</v>
-      </c>
-      <c r="O17" s="2">
-        <v>81</v>
-      </c>
-      <c r="P17">
-        <v>89.7</v>
-      </c>
-      <c r="R17" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S17" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T17" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U17">
-        <v>60</v>
-      </c>
-      <c r="V17" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="X17" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="J18" t="s">
-        <v>105</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>80</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="O18">
-        <v>91</v>
-      </c>
-      <c r="P18">
-        <v>89.6</v>
-      </c>
-      <c r="R18" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S18" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T18" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U18">
-        <v>60</v>
-      </c>
-      <c r="V18" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="X18" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19">
-        <v>1</v>
-      </c>
-      <c r="J19" t="s">
-        <v>105</v>
-      </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>100</v>
-      </c>
-      <c r="M19" t="s">
-        <v>79</v>
-      </c>
-      <c r="N19">
-        <v>5</v>
-      </c>
-      <c r="O19">
-        <v>90.7</v>
-      </c>
-      <c r="P19">
-        <v>89.65</v>
-      </c>
-      <c r="Q19">
-        <v>91.5</v>
-      </c>
-      <c r="R19" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S19" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T19" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U19">
-        <v>60</v>
-      </c>
-      <c r="V19" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="J20" t="s">
-        <v>105</v>
-      </c>
-      <c r="K20">
-        <v>2</v>
-      </c>
-      <c r="L20">
-        <v>90</v>
-      </c>
-      <c r="M20">
-        <v>34</v>
-      </c>
-      <c r="N20">
-        <v>5</v>
-      </c>
-      <c r="O20">
-        <v>91.6</v>
-      </c>
-      <c r="P20">
-        <v>89.6</v>
-      </c>
-      <c r="R20" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S20" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T20" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U20">
-        <v>60</v>
-      </c>
-      <c r="V20" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="X20" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="J21" t="s">
-        <v>105</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>100</v>
-      </c>
-      <c r="M21">
-        <v>7</v>
-      </c>
-      <c r="O21">
-        <v>91.5</v>
-      </c>
-      <c r="P21">
-        <v>89.6</v>
-      </c>
-      <c r="R21" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S21" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T21" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U21">
-        <v>60</v>
-      </c>
-      <c r="V21" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" t="s">
-        <v>98</v>
-      </c>
-      <c r="C22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="J22" t="s">
-        <v>105</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22">
-        <v>40</v>
-      </c>
-      <c r="M22" t="s">
-        <v>93</v>
-      </c>
-      <c r="O22">
-        <v>80</v>
-      </c>
-      <c r="P22">
-        <v>90.48</v>
-      </c>
-      <c r="Q22">
-        <v>84.7</v>
-      </c>
-      <c r="R22" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S22" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T22" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U22">
-        <v>30</v>
-      </c>
-      <c r="V22" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" t="s">
-        <v>98</v>
-      </c>
-      <c r="C23" t="s">
-        <v>92</v>
-      </c>
-      <c r="D23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E23">
-        <v>2</v>
-      </c>
-      <c r="J23" t="s">
-        <v>105</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
-        <v>53</v>
-      </c>
-      <c r="M23" t="s">
-        <v>94</v>
-      </c>
-      <c r="O23">
-        <v>79.8</v>
-      </c>
-      <c r="P23">
-        <v>90.56</v>
-      </c>
-      <c r="Q23">
-        <v>83.6</v>
-      </c>
-      <c r="R23" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S23" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T23" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U23">
-        <v>30</v>
-      </c>
-      <c r="V23" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" t="s">
-        <v>98</v>
-      </c>
-      <c r="C24" t="s">
-        <v>87</v>
-      </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="J24" t="s">
-        <v>105</v>
-      </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
-      <c r="L24">
-        <v>80</v>
-      </c>
-      <c r="M24" t="s">
+      <c r="W6" s="1">
+        <f>365*2</f>
+        <v>730</v>
+      </c>
+      <c r="Y6" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="O24">
-        <v>82.7</v>
-      </c>
-      <c r="P24" s="2">
-        <v>89.488135191811949</v>
-      </c>
-      <c r="Q24">
-        <v>85</v>
-      </c>
-      <c r="R24" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S24" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T24" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U24">
-        <v>60</v>
-      </c>
-      <c r="V24" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" t="s">
-        <v>98</v>
-      </c>
-      <c r="C25" t="s">
-        <v>91</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="J25" t="s">
-        <v>105</v>
-      </c>
-      <c r="K25">
-        <v>15</v>
-      </c>
-      <c r="L25">
-        <v>60</v>
-      </c>
-      <c r="M25">
-        <v>35.5</v>
-      </c>
-      <c r="O25">
-        <v>82.59</v>
-      </c>
-      <c r="P25">
-        <v>90.53</v>
-      </c>
-      <c r="R25" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S25" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T25" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U25">
-        <v>60</v>
-      </c>
-      <c r="V25" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B26" t="s">
-        <v>98</v>
-      </c>
-      <c r="C26" t="s">
-        <v>88</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="3"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="3"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="3"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="3"/>
+      <c r="V10" s="1"/>
+      <c r="W10" s="1"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="3"/>
+      <c r="V11" s="1"/>
+      <c r="W11" s="1"/>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
+      <c r="T12" s="3"/>
+      <c r="V12" s="1"/>
+      <c r="W12" s="1"/>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="3"/>
+      <c r="V13" s="1"/>
+      <c r="W13" s="1"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="3"/>
+      <c r="V14" s="1"/>
+      <c r="W14" s="1"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="O15" s="2"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="3"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="O16" s="2"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="3"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+    </row>
+    <row r="17" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="O17" s="2"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="3"/>
+      <c r="V17" s="1"/>
+      <c r="W17" s="1"/>
+    </row>
+    <row r="18" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="3"/>
+      <c r="V18" s="1"/>
+      <c r="W18" s="1"/>
+    </row>
+    <row r="19" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="3"/>
+      <c r="V19" s="1"/>
+      <c r="W19" s="1"/>
+    </row>
+    <row r="20" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="3"/>
+      <c r="V20" s="1"/>
+      <c r="W20" s="1"/>
+    </row>
+    <row r="21" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="3"/>
+      <c r="V21" s="1"/>
+      <c r="W21" s="1"/>
+    </row>
+    <row r="22" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="3"/>
+      <c r="V22" s="1"/>
+      <c r="W22" s="1"/>
+    </row>
+    <row r="23" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="3"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1"/>
+    </row>
+    <row r="24" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="P24" s="2"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="3"/>
+      <c r="V24" s="1"/>
+      <c r="W24" s="1"/>
+    </row>
+    <row r="25" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="3"/>
+      <c r="V25" s="1"/>
+      <c r="W25" s="1"/>
+    </row>
+    <row r="26" spans="5:23" x14ac:dyDescent="0.2">
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
-      <c r="J26" t="s">
-        <v>105</v>
-      </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-      <c r="L26">
-        <v>67</v>
-      </c>
-      <c r="M26">
-        <v>23</v>
-      </c>
-      <c r="O26">
-        <v>84.86</v>
-      </c>
-      <c r="P26">
-        <v>88.14</v>
-      </c>
-      <c r="R26" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S26" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T26" s="3">
-        <f t="shared" si="0"/>
-        <v>500000000</v>
-      </c>
-      <c r="U26">
-        <v>60</v>
-      </c>
-      <c r="V26" s="1">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="J27" t="s">
-        <v>105</v>
-      </c>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="3"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+    </row>
+    <row r="27" spans="5:23" x14ac:dyDescent="0.2">
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>83</v>
-      </c>
-      <c r="J28" t="s">
-        <v>105</v>
-      </c>
+    <row r="28" spans="5:23" x14ac:dyDescent="0.2">
       <c r="R28" s="1"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>82</v>
-      </c>
-      <c r="J29" t="s">
-        <v>105</v>
-      </c>
+    <row r="29" spans="5:23" x14ac:dyDescent="0.2">
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
       <c r="R29" s="1"/>
     </row>
-    <row r="30" spans="1:24" ht="51" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>96</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
-      </c>
-      <c r="J30" t="s">
-        <v>105</v>
-      </c>
-      <c r="K30">
-        <v>25</v>
-      </c>
-      <c r="L30">
-        <v>400</v>
-      </c>
-      <c r="M30">
-        <v>69</v>
-      </c>
-      <c r="O30">
-        <v>87</v>
-      </c>
-      <c r="P30">
-        <v>75.95</v>
-      </c>
-      <c r="R30" s="1">
-        <v>1250</v>
-      </c>
-      <c r="S30" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="T30" s="3">
-        <f t="shared" ref="T30" si="1">1000000000/2</f>
-        <v>500000000</v>
-      </c>
-      <c r="U30">
-        <v>600</v>
-      </c>
-      <c r="V30" s="1">
-        <v>2</v>
-      </c>
-      <c r="X30" s="7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="30" spans="5:23" x14ac:dyDescent="0.2">
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="3"/>
+      <c r="V30" s="1"/>
+      <c r="W30" s="1"/>
+    </row>
+    <row r="31" spans="5:23" x14ac:dyDescent="0.2">
       <c r="E31">
         <v>1</v>
       </c>
       <c r="V31" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B32" t="s">
-        <v>111</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E32">
-        <v>1</v>
-      </c>
-      <c r="F32" s="9">
-        <v>88</v>
-      </c>
-      <c r="G32" s="10">
-        <v>123</v>
-      </c>
-      <c r="H32" s="11">
-        <v>33</v>
-      </c>
-      <c r="J32" t="s">
-        <v>68</v>
-      </c>
-      <c r="K32" s="13">
-        <v>0</v>
-      </c>
-      <c r="L32" s="13">
-        <v>300</v>
-      </c>
-      <c r="M32" s="13">
-        <v>46</v>
-      </c>
-      <c r="O32" s="13">
-        <v>82</v>
-      </c>
-      <c r="P32" s="13">
-        <v>88.5</v>
-      </c>
-      <c r="R32">
-        <v>1200</v>
-      </c>
-      <c r="S32">
-        <f xml:space="preserve"> 100000 * 10^-7.86</f>
-        <v>1.3803842646028805E-3</v>
-      </c>
-      <c r="T32" s="8">
-        <f>42*10^6</f>
-        <v>42000000</v>
-      </c>
-      <c r="U32">
-        <v>600</v>
-      </c>
-      <c r="V32" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:24" ht="136" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B33" t="s">
-        <v>111</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E33">
-        <v>1</v>
-      </c>
-      <c r="F33" s="9">
-        <v>81</v>
-      </c>
-      <c r="G33" s="10">
-        <v>166</v>
-      </c>
-      <c r="H33" s="11">
-        <v>79</v>
-      </c>
-      <c r="J33" t="s">
-        <v>68</v>
-      </c>
-      <c r="K33" s="13">
-        <v>0</v>
-      </c>
-      <c r="L33" s="13">
-        <v>190</v>
-      </c>
-      <c r="M33">
-        <v>40</v>
-      </c>
-      <c r="O33">
-        <v>82</v>
-      </c>
-      <c r="P33">
-        <v>87.8</v>
-      </c>
-      <c r="R33">
-        <v>1200</v>
-      </c>
-      <c r="S33">
-        <f t="shared" ref="S33:S34" si="2" xml:space="preserve"> 100000 * 10^-7.86</f>
-        <v>1.3803842646028805E-3</v>
-      </c>
-      <c r="T33" s="8">
-        <f t="shared" ref="T33:T36" si="3">42*10^6</f>
-        <v>42000000</v>
-      </c>
-      <c r="U33">
-        <v>600</v>
-      </c>
-      <c r="V33" s="1">
-        <v>1</v>
-      </c>
-      <c r="X33" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="34" spans="1:24" ht="204" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B34" t="s">
-        <v>111</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E34">
-        <v>1</v>
-      </c>
-      <c r="F34" s="9">
-        <v>119</v>
-      </c>
-      <c r="G34" s="10">
-        <v>110</v>
-      </c>
-      <c r="H34" s="11">
-        <v>37</v>
-      </c>
-      <c r="J34" t="s">
-        <v>68</v>
-      </c>
-      <c r="K34" s="13">
-        <v>0</v>
-      </c>
-      <c r="L34" s="13">
-        <v>300</v>
-      </c>
-      <c r="M34" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="O34" s="2">
-        <v>82.6</v>
-      </c>
-      <c r="P34">
-        <v>85.9</v>
-      </c>
-      <c r="Q34">
-        <v>88.5</v>
-      </c>
-      <c r="R34">
-        <v>1200</v>
-      </c>
-      <c r="S34">
-        <f t="shared" si="2"/>
-        <v>1.3803842646028805E-3</v>
-      </c>
-      <c r="T34" s="8">
-        <f t="shared" si="3"/>
-        <v>42000000</v>
-      </c>
-      <c r="U34">
-        <v>600</v>
-      </c>
-      <c r="V34" s="1">
-        <v>1</v>
-      </c>
-      <c r="X34" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B35" t="s">
-        <v>111</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35" s="9">
-        <v>60</v>
-      </c>
-      <c r="G35" s="10">
-        <v>30</v>
-      </c>
-      <c r="H35" s="11">
-        <v>90</v>
-      </c>
-      <c r="J35" t="s">
-        <v>68</v>
-      </c>
-      <c r="K35" s="13">
-        <v>0</v>
-      </c>
-      <c r="L35" s="13">
-        <v>150</v>
-      </c>
-      <c r="M35" t="s">
-        <v>117</v>
-      </c>
-      <c r="O35">
-        <v>67</v>
-      </c>
-      <c r="P35">
-        <v>60.5</v>
-      </c>
-      <c r="Q35">
-        <v>73.5</v>
-      </c>
-      <c r="R35" s="12">
-        <v>1102</v>
-      </c>
-      <c r="S35">
-        <f xml:space="preserve"> 100000 * 10^-8.74</f>
-        <v>1.8197008586099805E-4</v>
-      </c>
-      <c r="T35" s="8">
-        <f t="shared" si="3"/>
-        <v>42000000</v>
-      </c>
-      <c r="U35">
-        <v>600</v>
-      </c>
-      <c r="V35" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B36" t="s">
-        <v>111</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" s="9">
-        <v>89</v>
-      </c>
-      <c r="G36" s="10">
-        <v>3</v>
-      </c>
-      <c r="H36" s="11">
-        <v>88</v>
-      </c>
-      <c r="J36" t="s">
-        <v>68</v>
-      </c>
-      <c r="R36" s="12">
-        <v>1102</v>
-      </c>
-      <c r="S36">
-        <f xml:space="preserve"> 100000 * 10^-8.74</f>
-        <v>1.8197008586099805E-4</v>
-      </c>
-      <c r="T36" s="8">
-        <f t="shared" si="3"/>
-        <v>42000000</v>
-      </c>
-      <c r="U36">
-        <v>600</v>
-      </c>
-      <c r="V36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="W31" s="1"/>
+    </row>
+    <row r="39" spans="11:16" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="P39" s="1"/>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="47" spans="11:16" x14ac:dyDescent="0.2">
       <c r="M47" s="5"/>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="48" spans="11:16" x14ac:dyDescent="0.2">
       <c r="M48" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="O15:O17">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
-      <formula>83</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O34">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
-      <formula>83</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3841,7 +2738,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="O15">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="lessThan">
       <formula>83</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
-Krige Interpolation Uncertainty Finalized - Output table developed and formated using Great Tables
</commit_message>
<xml_diff>
--- a/Diffusion Round Robin/Round_Robin_Olivine_Profile_Diffusion_Modeling_Parameters_DB.xlsx
+++ b/Diffusion Round Robin/Round_Robin_Olivine_Profile_Diffusion_Modeling_Parameters_DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henrytowbin/Projects/Olivine_Diffusion_FeMg/Diffusion Round Robin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DE563E-AC8C-4048-99A0-D5C31D62B8EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED77917-DEA3-C443-A9E9-18C69FACBC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4760" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{4BF80DE2-54EF-754E-B733-C83BF6E05191}"/>
+    <workbookView xWindow="-560" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{4BF80DE2-54EF-754E-B733-C83BF6E05191}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="144">
   <si>
     <t>Sample</t>
   </si>
@@ -313,15 +313,9 @@
     <t>Hard to say where the multiple steps should be. Inflection closest most could be at 0,  20, or ~40µm, CaO would suggest 40µm. Next inflection could be ~90 - 100 µm based on 1st derivative flattening and MnO  and CaO changing shape. Based on profile shape it could be as far as 150µm, max concentration is unknown. I should model 3 ways, highest measured in all 3 samples, next highest measured in samples  then highest in this sample</t>
   </si>
   <si>
-    <t>1, 100</t>
-  </si>
-  <si>
     <t>Could be modeled with same initial as previous. Inflection at 50µm based on the first and second derivative  of Fo.  MnO, and CaO suggest it should be between 40 and 50. The flat profiles in Mn and Ca might suggest growth and not diffusion, Model Can also be fit with no inflection point</t>
   </si>
   <si>
-    <t>0, 20</t>
-  </si>
-  <si>
     <t>P isnt too useful for determining the step position. The derivative  of the smoothed data is more useful.</t>
   </si>
   <si>
@@ -404,6 +398,78 @@
   </si>
   <si>
     <t>Uncert_Category</t>
+  </si>
+  <si>
+    <t>KS20-527_2-transect-4</t>
+  </si>
+  <si>
+    <t>SH63olv066-3</t>
+  </si>
+  <si>
+    <t>SH63olv066-4</t>
+  </si>
+  <si>
+    <t>0, 21</t>
+  </si>
+  <si>
+    <t>Descriptive_Name</t>
+  </si>
+  <si>
+    <t>Step 42µm</t>
+  </si>
+  <si>
+    <t>Step 41µm</t>
+  </si>
+  <si>
+    <t>Step 46µm</t>
+  </si>
+  <si>
+    <t>Step 51µm</t>
+  </si>
+  <si>
+    <t>Step 40µm</t>
+  </si>
+  <si>
+    <t>Step 50µm</t>
+  </si>
+  <si>
+    <t>Step 55µm</t>
+  </si>
+  <si>
+    <t>yes+K13</t>
+  </si>
+  <si>
+    <t>0, 100</t>
+  </si>
+  <si>
+    <t>Step 0 and 100µm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 0 and 121µm, Edge Fo67 Peak Fo74.5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 0 and 145µm, Peak Fo87.2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 0 and 120µm, Peak Fo87.8 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 35 and 120µm, Peak Fo87.8 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 20 and 100µm, Peak Fo88.5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 0 and 121µm, Edge Fo69 Peak Fo74.5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 0 and 121µm, Edge Fo68 Peak Fo74.5 </t>
+  </si>
+  <si>
+    <t>No Step</t>
+  </si>
+  <si>
+    <t>Step 0 and 121µm, Edge Fo69 Peak Fo74</t>
   </si>
 </sst>
 </file>
@@ -856,1214 +922,1467 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D2757E0-7F0F-D849-AAD1-AAB451BA4D11}">
-  <dimension ref="A1:Z57"/>
+  <dimension ref="A1:AA60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.5" customWidth="1"/>
-    <col min="3" max="3" width="38.1640625" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="17.33203125" customWidth="1"/>
-    <col min="14" max="14" width="21.5" customWidth="1"/>
-    <col min="17" max="17" width="16.6640625" customWidth="1"/>
-    <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="21.5" customWidth="1"/>
-    <col min="24" max="24" width="21.33203125" customWidth="1"/>
-    <col min="25" max="25" width="36.1640625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="32.5" customWidth="1"/>
+    <col min="4" max="4" width="38.1640625" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="17.33203125" customWidth="1"/>
+    <col min="15" max="15" width="21.5" customWidth="1"/>
+    <col min="18" max="18" width="16.6640625" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
+    <col min="22" max="22" width="21.5" customWidth="1"/>
+    <col min="25" max="25" width="21.33203125" customWidth="1"/>
+    <col min="26" max="26" width="36.1640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
-        <v>121</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>82</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>67</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>95</v>
       </c>
       <c r="X1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="9">
+      <c r="E2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9">
         <v>88</v>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="10">
         <v>123</v>
       </c>
-      <c r="H2" s="11">
+      <c r="I2" s="11">
         <v>33</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>68</v>
       </c>
-      <c r="K2" s="13">
+      <c r="L2" s="13">
         <v>0</v>
       </c>
-      <c r="L2" s="13">
+      <c r="M2" s="13">
         <v>300</v>
       </c>
-      <c r="M2" s="13">
+      <c r="N2" s="13">
         <v>41</v>
       </c>
-      <c r="O2" s="13">
+      <c r="P2" s="13">
         <v>82</v>
       </c>
-      <c r="P2" s="13">
+      <c r="Q2" s="13">
         <v>88.5</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>1200</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <f xml:space="preserve"> 100000 * 10^-7.86</f>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T2" s="8">
+      <c r="U2" s="8">
         <f>42*10^6</f>
         <v>42000000</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>600</v>
       </c>
-      <c r="V2" s="1">
-        <v>1</v>
-      </c>
-      <c r="W2" s="1"/>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="W2" s="1">
+        <v>1</v>
+      </c>
+      <c r="X2" s="1"/>
+    </row>
+    <row r="3" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" s="9">
+      <c r="E3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="9">
         <v>88</v>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="10">
         <v>123</v>
       </c>
-      <c r="H3" s="11">
+      <c r="I3" s="11">
         <v>33</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>68</v>
       </c>
-      <c r="K3" s="13">
+      <c r="L3" s="13">
         <v>0</v>
       </c>
-      <c r="L3" s="13">
+      <c r="M3" s="13">
         <v>300</v>
       </c>
-      <c r="M3" s="13">
-        <v>46</v>
-      </c>
-      <c r="O3" s="13">
+      <c r="N3" s="13">
+        <v>42</v>
+      </c>
+      <c r="P3" s="13">
         <v>82</v>
       </c>
-      <c r="P3" s="13">
+      <c r="Q3" s="13">
         <v>88.5</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>1200</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <f xml:space="preserve"> 100000 * 10^-7.86</f>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T3" s="8">
+      <c r="U3" s="8">
         <f>42*10^6</f>
         <v>42000000</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>600</v>
       </c>
-      <c r="V3" s="1">
-        <v>1</v>
-      </c>
-      <c r="W3" s="1"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="W3" s="1">
+        <v>1</v>
+      </c>
+      <c r="X3" s="1"/>
+    </row>
+    <row r="4" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" t="s">
         <v>115</v>
       </c>
-      <c r="B4" t="s">
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="9">
         <v>88</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" s="9">
-        <v>88</v>
-      </c>
-      <c r="G4" s="10">
+      <c r="H4" s="10">
         <v>123</v>
       </c>
-      <c r="H4" s="11">
+      <c r="I4" s="11">
         <v>33</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="13">
+      <c r="L4" s="13">
         <v>0</v>
       </c>
-      <c r="L4" s="13">
+      <c r="M4" s="13">
         <v>300</v>
       </c>
-      <c r="M4" s="13">
-        <v>51</v>
-      </c>
-      <c r="O4" s="13">
+      <c r="N4" s="13">
+        <v>46</v>
+      </c>
+      <c r="P4" s="13">
         <v>82</v>
       </c>
-      <c r="P4" s="13">
+      <c r="Q4" s="13">
         <v>88.5</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>1200</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <f xml:space="preserve"> 100000 * 10^-7.86</f>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T4" s="8">
+      <c r="U4" s="8">
         <f>42*10^6</f>
         <v>42000000</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>600</v>
       </c>
-      <c r="V4" s="1">
-        <v>1</v>
-      </c>
-      <c r="W4" s="1"/>
-    </row>
-    <row r="5" spans="1:26" ht="136" x14ac:dyDescent="0.2">
+      <c r="W4" s="1">
+        <v>1</v>
+      </c>
+      <c r="X4" s="1"/>
+    </row>
+    <row r="5" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="9">
+        <v>88</v>
+      </c>
+      <c r="H5" s="10">
+        <v>123</v>
+      </c>
+      <c r="I5" s="11">
+        <v>33</v>
+      </c>
+      <c r="K5" t="s">
+        <v>68</v>
+      </c>
+      <c r="L5" s="13">
+        <v>0</v>
+      </c>
+      <c r="M5" s="13">
+        <v>300</v>
+      </c>
+      <c r="N5" s="13">
+        <v>51</v>
+      </c>
+      <c r="P5" s="13">
+        <v>82</v>
+      </c>
+      <c r="Q5" s="13">
+        <v>88.5</v>
+      </c>
+      <c r="S5">
+        <v>1200</v>
+      </c>
+      <c r="T5">
+        <f xml:space="preserve"> 100000 * 10^-7.86</f>
+        <v>1.3803842646028805E-3</v>
+      </c>
+      <c r="U5" s="8">
+        <f>42*10^6</f>
+        <v>42000000</v>
+      </c>
+      <c r="V5">
+        <v>600</v>
+      </c>
+      <c r="W5" s="1">
+        <v>1</v>
+      </c>
+      <c r="X5" s="1"/>
+    </row>
+    <row r="6" spans="1:27" ht="136" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" s="9">
+      <c r="E6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9">
         <v>81</v>
       </c>
-      <c r="G5" s="10">
+      <c r="H6" s="10">
         <v>166</v>
       </c>
-      <c r="H5" s="11">
+      <c r="I6" s="11">
         <v>79</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K6" t="s">
         <v>68</v>
       </c>
-      <c r="K5" s="13">
+      <c r="L6" s="13">
         <v>0</v>
       </c>
-      <c r="L5" s="13">
+      <c r="M6" s="13">
         <v>190</v>
       </c>
-      <c r="M5">
+      <c r="N6">
         <v>40</v>
       </c>
-      <c r="O5">
+      <c r="P6">
         <v>82.4</v>
       </c>
-      <c r="P5">
+      <c r="Q6">
         <v>87.8</v>
       </c>
-      <c r="R5">
+      <c r="S6">
         <v>1200</v>
       </c>
-      <c r="S5">
-        <f t="shared" ref="S5:S12" si="0" xml:space="preserve"> 100000 * 10^-7.86</f>
+      <c r="T6">
+        <f t="shared" ref="T6:T13" si="0" xml:space="preserve"> 100000 * 10^-7.86</f>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T5" s="8">
-        <f t="shared" ref="T5:T12" si="1">42*10^6</f>
+      <c r="U6" s="8">
+        <f t="shared" ref="U6:U13" si="1">42*10^6</f>
         <v>42000000</v>
       </c>
-      <c r="U5">
+      <c r="V6">
         <v>600</v>
       </c>
-      <c r="V5" s="1">
-        <v>1</v>
-      </c>
-      <c r="W5" s="1"/>
-      <c r="Y5" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="136" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="W6" s="1">
+        <v>1</v>
+      </c>
+      <c r="X6" s="1"/>
+      <c r="Z6" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="136" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" s="9">
+      <c r="E7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" s="9">
         <v>81</v>
       </c>
-      <c r="G6" s="10">
+      <c r="H7" s="10">
         <v>166</v>
       </c>
-      <c r="H6" s="11">
+      <c r="I7" s="11">
         <v>79</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K7" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="13">
+      <c r="L7" s="13">
         <v>0</v>
       </c>
-      <c r="L6" s="13">
+      <c r="M7" s="13">
         <v>190</v>
       </c>
-      <c r="M6">
+      <c r="N7">
         <v>50</v>
       </c>
-      <c r="O6">
+      <c r="P7">
         <v>82.4</v>
       </c>
-      <c r="P6">
+      <c r="Q7">
         <v>87.8</v>
       </c>
-      <c r="R6">
+      <c r="S7">
         <v>1200</v>
       </c>
-      <c r="S6">
+      <c r="T7">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T6" s="8">
+      <c r="U7" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U6">
+      <c r="V7">
         <v>600</v>
       </c>
-      <c r="V6" s="1">
-        <v>1</v>
-      </c>
-      <c r="W6" s="1"/>
-      <c r="Y6" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="136" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="W7" s="1">
+        <v>1</v>
+      </c>
+      <c r="X7" s="1"/>
+      <c r="Z7" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="136" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D7" t="s">
-        <v>117</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" s="9">
+      <c r="E8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="9">
         <v>81</v>
       </c>
-      <c r="G7" s="10">
+      <c r="H8" s="10">
         <v>166</v>
       </c>
-      <c r="H7" s="11">
+      <c r="I8" s="11">
         <v>79</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K8" t="s">
         <v>68</v>
       </c>
-      <c r="K7" s="13">
+      <c r="L8" s="13">
         <v>0</v>
       </c>
-      <c r="L7" s="13">
+      <c r="M8" s="13">
         <v>190</v>
       </c>
-      <c r="M7">
+      <c r="N8">
         <v>55</v>
       </c>
-      <c r="O7">
+      <c r="P8">
         <v>82.4</v>
       </c>
-      <c r="P7">
+      <c r="Q8">
         <v>87.8</v>
       </c>
-      <c r="R7">
+      <c r="S8">
         <v>1200</v>
       </c>
-      <c r="S7">
+      <c r="T8">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T7" s="8">
+      <c r="U8" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U7">
+      <c r="V8">
         <v>600</v>
       </c>
-      <c r="V7" s="1">
-        <v>1</v>
-      </c>
-      <c r="W7" s="1"/>
-      <c r="Y7" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="204" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="W8" s="1">
+        <v>1</v>
+      </c>
+      <c r="X8" s="1"/>
+      <c r="Z8" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="204" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D8" t="s">
-        <v>117</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" s="9">
+      <c r="E9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" s="9">
         <v>119</v>
       </c>
-      <c r="G8" s="10">
+      <c r="H9" s="10">
         <v>110</v>
       </c>
-      <c r="H8" s="11">
+      <c r="I9" s="11">
         <v>37</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K9" t="s">
         <v>68</v>
       </c>
-      <c r="K8" s="13">
+      <c r="L9" s="13">
         <v>0</v>
       </c>
-      <c r="L8" s="13">
+      <c r="M9" s="13">
         <v>300</v>
       </c>
-      <c r="M8" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="O8" s="2">
+      <c r="N9" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="P9" s="2">
         <v>82.6</v>
       </c>
-      <c r="P8">
+      <c r="Q9">
         <v>85.9</v>
       </c>
-      <c r="Q8">
+      <c r="R9">
         <v>88.5</v>
       </c>
-      <c r="R8">
+      <c r="S9">
         <v>1200</v>
       </c>
-      <c r="S8">
+      <c r="T9">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T8" s="8">
+      <c r="U9" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U8">
+      <c r="V9">
         <v>600</v>
       </c>
-      <c r="V8" s="1">
-        <v>1</v>
-      </c>
-      <c r="W8" s="1"/>
-      <c r="Y8" s="7" t="s">
+      <c r="W9" s="1">
+        <v>1</v>
+      </c>
+      <c r="X9" s="1"/>
+      <c r="Z9" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="204" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:27" ht="204" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" s="9">
+        <v>119</v>
+      </c>
+      <c r="H10" s="10">
+        <v>110</v>
+      </c>
+      <c r="I10" s="11">
+        <v>37</v>
+      </c>
+      <c r="K10" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="13">
+        <v>0</v>
+      </c>
+      <c r="M10" s="13">
+        <v>300</v>
+      </c>
+      <c r="N10" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" s="9">
-        <v>119</v>
-      </c>
-      <c r="G9" s="10">
-        <v>110</v>
-      </c>
-      <c r="H9" s="11">
-        <v>37</v>
-      </c>
-      <c r="J9" t="s">
-        <v>68</v>
-      </c>
-      <c r="K9" s="13">
-        <v>0</v>
-      </c>
-      <c r="L9" s="13">
-        <v>300</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="O9" s="2">
+      <c r="P10" s="2">
         <v>82.6</v>
       </c>
-      <c r="P9">
+      <c r="Q10">
         <v>85.9</v>
       </c>
-      <c r="Q9">
+      <c r="R10">
         <v>88.5</v>
       </c>
-      <c r="R9">
+      <c r="S10">
         <v>1200</v>
       </c>
-      <c r="S9">
+      <c r="T10">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T9" s="8">
+      <c r="U10" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U9">
+      <c r="V10">
         <v>600</v>
       </c>
-      <c r="V9" s="1">
-        <v>1</v>
-      </c>
-      <c r="W9" s="1"/>
-      <c r="Y9" s="7" t="s">
+      <c r="W10" s="1">
+        <v>1</v>
+      </c>
+      <c r="X10" s="1"/>
+      <c r="Z10" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="204" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B10" t="s">
+    <row r="11" spans="1:27" ht="204" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D10" t="s">
-        <v>117</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" s="9">
+      <c r="E11" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" s="9">
         <v>119</v>
       </c>
-      <c r="G10" s="10">
+      <c r="H11" s="10">
         <v>110</v>
       </c>
-      <c r="H10" s="11">
+      <c r="I11" s="11">
         <v>37</v>
       </c>
-      <c r="J10" t="s">
-        <v>68</v>
-      </c>
-      <c r="K10" s="13">
+      <c r="K11" t="s">
+        <v>132</v>
+      </c>
+      <c r="L11" s="13">
         <v>0</v>
       </c>
-      <c r="L10" s="13">
+      <c r="M11" s="13">
         <v>300</v>
       </c>
-      <c r="M10" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="O10" s="2">
+      <c r="N11" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="P11" s="2">
         <v>82.6</v>
       </c>
-      <c r="P10">
+      <c r="Q11">
         <v>85.9</v>
       </c>
-      <c r="Q10">
+      <c r="R11">
         <v>87.8</v>
       </c>
-      <c r="R10">
+      <c r="S11">
         <v>1200</v>
       </c>
-      <c r="S10">
+      <c r="T11">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T10" s="8">
+      <c r="U11" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U10">
+      <c r="V11">
         <v>600</v>
       </c>
-      <c r="V10" s="1">
-        <v>1</v>
-      </c>
-      <c r="W10" s="1"/>
-      <c r="Y10" s="7" t="s">
+      <c r="W11" s="1">
+        <v>1</v>
+      </c>
+      <c r="X11" s="1"/>
+      <c r="Z11" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="204" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" t="s">
+    <row r="12" spans="1:27" ht="204" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C12" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D11" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9">
+      <c r="E12" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="9">
         <v>119</v>
       </c>
-      <c r="G11" s="10">
+      <c r="H12" s="10">
         <v>110</v>
       </c>
-      <c r="H11" s="11">
+      <c r="I12" s="11">
         <v>37</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K12" t="s">
         <v>68</v>
       </c>
-      <c r="K11" s="13">
+      <c r="L12" s="13">
         <v>0</v>
       </c>
-      <c r="L11" s="13">
+      <c r="M12" s="13">
         <v>300</v>
       </c>
-      <c r="M11" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="O11" s="2">
+      <c r="N12" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="P12" s="2">
         <v>82.6</v>
       </c>
-      <c r="P11">
+      <c r="Q12">
         <v>85.9</v>
       </c>
-      <c r="Q11">
+      <c r="R12">
         <v>87.8</v>
       </c>
-      <c r="R11">
+      <c r="S12">
         <v>1200</v>
       </c>
-      <c r="S11">
+      <c r="T12">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T11" s="8">
+      <c r="U12" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U11">
+      <c r="V12">
         <v>600</v>
       </c>
-      <c r="V11" s="1">
-        <v>1</v>
-      </c>
-      <c r="W11" s="1"/>
-      <c r="Y11" s="7" t="s">
+      <c r="W12" s="1">
+        <v>1</v>
+      </c>
+      <c r="X12" s="1"/>
+      <c r="Z12" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="204" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:27" ht="204" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" s="9">
         <v>119</v>
       </c>
-      <c r="B12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" s="9">
-        <v>119</v>
-      </c>
-      <c r="G12" s="10">
+      <c r="H13" s="10">
         <v>110</v>
       </c>
-      <c r="H12" s="11">
+      <c r="I13" s="11">
         <v>37</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K13" t="s">
         <v>68</v>
       </c>
-      <c r="K12" s="13">
+      <c r="L13" s="13">
         <v>0</v>
       </c>
-      <c r="L12" s="13">
+      <c r="M13" s="13">
         <v>300</v>
       </c>
-      <c r="M12" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="O12" s="2">
+      <c r="N13" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="P13" s="2">
         <v>82.6</v>
       </c>
-      <c r="P12">
+      <c r="Q13">
         <v>85.9</v>
       </c>
-      <c r="Q12">
+      <c r="R13">
         <v>87.2</v>
       </c>
-      <c r="R12">
+      <c r="S13">
         <v>1200</v>
       </c>
-      <c r="S12">
+      <c r="T13">
         <f t="shared" si="0"/>
         <v>1.3803842646028805E-3</v>
       </c>
-      <c r="T12" s="8">
+      <c r="U13" s="8">
         <f t="shared" si="1"/>
         <v>42000000</v>
       </c>
-      <c r="U12">
+      <c r="V13">
         <v>600</v>
       </c>
-      <c r="V12" s="1">
-        <v>1</v>
-      </c>
-      <c r="W12" s="1"/>
-      <c r="Y12" s="7" t="s">
+      <c r="W13" s="1">
+        <v>1</v>
+      </c>
+      <c r="X13" s="1"/>
+      <c r="Z13" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="14" spans="1:27" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D13" t="s">
-        <v>118</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13" s="9">
+      <c r="E14" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="9">
         <v>60</v>
       </c>
-      <c r="G13" s="10">
+      <c r="H14" s="10">
         <v>30</v>
       </c>
-      <c r="H13" s="11">
+      <c r="I14" s="11">
         <v>90</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K14" t="s">
         <v>68</v>
       </c>
-      <c r="K13" s="13">
+      <c r="L14" s="13">
         <v>0</v>
       </c>
-      <c r="L13" s="13">
+      <c r="M14" s="13">
         <v>150</v>
       </c>
-      <c r="M13" t="s">
-        <v>93</v>
-      </c>
-      <c r="O13">
+      <c r="N14" t="s">
+        <v>123</v>
+      </c>
+      <c r="P14">
         <v>67</v>
       </c>
-      <c r="P13">
+      <c r="Q14">
         <v>60.5</v>
       </c>
-      <c r="Q13">
+      <c r="R14">
         <v>74.5</v>
       </c>
-      <c r="R13" s="12">
+      <c r="S14" s="12">
         <v>1102</v>
       </c>
-      <c r="S13">
+      <c r="T14">
         <f xml:space="preserve"> 100000 * 10^-8.74</f>
         <v>1.8197008586099805E-4</v>
       </c>
-      <c r="T13" s="8">
+      <c r="U14" s="8">
         <f>70*10^6</f>
         <v>70000000</v>
       </c>
-      <c r="U13">
+      <c r="V14">
         <v>120</v>
       </c>
-      <c r="V13" s="1">
-        <v>1</v>
-      </c>
-      <c r="W13" s="1"/>
-      <c r="Y13" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="W14" s="1">
+        <v>1</v>
+      </c>
+      <c r="X14" s="1"/>
+      <c r="Z14" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D14" t="s">
-        <v>118</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14" s="9">
+      <c r="E15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" s="9">
         <v>60</v>
       </c>
-      <c r="G14" s="10">
+      <c r="H15" s="10">
         <v>30</v>
       </c>
-      <c r="H14" s="11">
+      <c r="I15" s="11">
         <v>90</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K15" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="13">
+      <c r="L15" s="13">
         <v>0</v>
       </c>
-      <c r="L14" s="13">
+      <c r="M15" s="13">
         <v>150</v>
       </c>
-      <c r="M14" t="s">
-        <v>93</v>
-      </c>
-      <c r="O14">
-        <v>67</v>
-      </c>
-      <c r="P14">
+      <c r="N15" t="s">
+        <v>123</v>
+      </c>
+      <c r="P15">
+        <v>68</v>
+      </c>
+      <c r="Q15">
         <v>60.5</v>
       </c>
-      <c r="Q14">
-        <v>74</v>
-      </c>
-      <c r="R14" s="12">
+      <c r="R15">
+        <v>74.5</v>
+      </c>
+      <c r="S15" s="12">
         <v>1102</v>
       </c>
-      <c r="S14">
+      <c r="T15">
         <f xml:space="preserve"> 100000 * 10^-8.74</f>
         <v>1.8197008586099805E-4</v>
       </c>
-      <c r="T14" s="8">
-        <f t="shared" ref="T14:T15" si="2">70*10^6</f>
+      <c r="U15" s="8">
+        <f t="shared" ref="U15:U18" si="2">70*10^6</f>
         <v>70000000</v>
       </c>
-      <c r="U14">
+      <c r="V15">
         <v>120</v>
       </c>
-      <c r="V14" s="1">
-        <v>1</v>
-      </c>
-      <c r="W14" s="1"/>
-      <c r="Y14" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="68" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="W15" s="1">
+        <v>1</v>
+      </c>
+      <c r="X15" s="1"/>
+      <c r="Z15" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" ht="51" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" t="s">
-        <v>118</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="F15" s="9">
-        <v>89</v>
-      </c>
-      <c r="G15" s="10">
-        <v>3</v>
-      </c>
-      <c r="H15" s="11">
-        <v>88</v>
-      </c>
-      <c r="J15" t="s">
+      <c r="D16" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" s="9">
+        <v>60</v>
+      </c>
+      <c r="H16" s="10">
+        <v>30</v>
+      </c>
+      <c r="I16" s="11">
+        <v>90</v>
+      </c>
+      <c r="K16" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="13">
+      <c r="L16" s="13">
         <v>0</v>
       </c>
-      <c r="L15" s="13">
-        <v>160</v>
-      </c>
-      <c r="M15" s="13">
-        <v>0</v>
-      </c>
-      <c r="O15">
-        <v>73</v>
-      </c>
-      <c r="P15">
-        <v>62.6</v>
-      </c>
-      <c r="R15" s="12">
+      <c r="M16" s="13">
+        <v>150</v>
+      </c>
+      <c r="N16" t="s">
+        <v>123</v>
+      </c>
+      <c r="P16">
+        <v>69</v>
+      </c>
+      <c r="Q16">
+        <v>60.5</v>
+      </c>
+      <c r="R16">
+        <v>74.5</v>
+      </c>
+      <c r="S16" s="12">
         <v>1102</v>
       </c>
-      <c r="S15">
+      <c r="T16">
         <f xml:space="preserve"> 100000 * 10^-8.74</f>
         <v>1.8197008586099805E-4</v>
       </c>
-      <c r="T15" s="8">
+      <c r="U16" s="8">
         <f t="shared" si="2"/>
         <v>70000000</v>
       </c>
-      <c r="U15">
+      <c r="V16">
+        <v>120</v>
+      </c>
+      <c r="W16" s="1">
+        <v>1</v>
+      </c>
+      <c r="X16" s="1"/>
+      <c r="Z16" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" s="9">
+        <v>60</v>
+      </c>
+      <c r="H17" s="10">
+        <v>30</v>
+      </c>
+      <c r="I17" s="11">
+        <v>90</v>
+      </c>
+      <c r="K17" t="s">
+        <v>68</v>
+      </c>
+      <c r="L17" s="13">
+        <v>0</v>
+      </c>
+      <c r="M17" s="13">
+        <v>150</v>
+      </c>
+      <c r="N17" t="s">
+        <v>123</v>
+      </c>
+      <c r="P17">
+        <v>69</v>
+      </c>
+      <c r="Q17">
+        <v>60.5</v>
+      </c>
+      <c r="R17">
+        <v>74</v>
+      </c>
+      <c r="S17" s="12">
+        <v>1102</v>
+      </c>
+      <c r="T17">
+        <f xml:space="preserve"> 100000 * 10^-8.74</f>
+        <v>1.8197008586099805E-4</v>
+      </c>
+      <c r="U17" s="8">
+        <f t="shared" si="2"/>
+        <v>70000000</v>
+      </c>
+      <c r="V17">
+        <v>120</v>
+      </c>
+      <c r="W17" s="1">
+        <v>1</v>
+      </c>
+      <c r="X17" s="1"/>
+      <c r="Z17" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" ht="68" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" s="9">
+        <v>89</v>
+      </c>
+      <c r="H18" s="10">
+        <v>3</v>
+      </c>
+      <c r="I18" s="11">
+        <v>88</v>
+      </c>
+      <c r="K18" t="s">
+        <v>68</v>
+      </c>
+      <c r="L18" s="13">
+        <v>0</v>
+      </c>
+      <c r="M18" s="13">
+        <v>160</v>
+      </c>
+      <c r="N18" s="13">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>73</v>
+      </c>
+      <c r="Q18">
+        <v>62.6</v>
+      </c>
+      <c r="S18" s="12">
+        <v>1102</v>
+      </c>
+      <c r="T18">
+        <f xml:space="preserve"> 100000 * 10^-8.74</f>
+        <v>1.8197008586099805E-4</v>
+      </c>
+      <c r="U18" s="8">
+        <f t="shared" si="2"/>
+        <v>70000000</v>
+      </c>
+      <c r="V18">
         <v>600</v>
       </c>
-      <c r="V15" s="1">
-        <v>1</v>
-      </c>
-      <c r="W15" s="1">
+      <c r="W18" s="1">
+        <v>1</v>
+      </c>
+      <c r="X18" s="1">
         <f>365*2</f>
         <v>730</v>
       </c>
-      <c r="Y15" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="3"/>
-      <c r="V16" s="1"/>
-      <c r="W16" s="1"/>
-    </row>
-    <row r="17" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="3"/>
-      <c r="V17" s="1"/>
-      <c r="W17" s="1"/>
-    </row>
-    <row r="18" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="3"/>
-      <c r="V18" s="1"/>
-      <c r="W18" s="1"/>
-    </row>
-    <row r="19" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R19" s="1"/>
+      <c r="Z18" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S19" s="1"/>
-      <c r="T19" s="3"/>
-      <c r="V19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="3"/>
       <c r="W19" s="1"/>
-    </row>
-    <row r="20" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R20" s="1"/>
+      <c r="X19" s="1"/>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S20" s="1"/>
-      <c r="T20" s="3"/>
-      <c r="V20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="3"/>
       <c r="W20" s="1"/>
-    </row>
-    <row r="21" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R21" s="1"/>
+      <c r="X20" s="1"/>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S21" s="1"/>
-      <c r="T21" s="3"/>
-      <c r="V21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="3"/>
       <c r="W21" s="1"/>
-    </row>
-    <row r="22" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R22" s="1"/>
+      <c r="X21" s="1"/>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S22" s="1"/>
-      <c r="T22" s="3"/>
-      <c r="V22" s="1"/>
+      <c r="T22" s="1"/>
+      <c r="U22" s="3"/>
       <c r="W22" s="1"/>
-    </row>
-    <row r="23" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R23" s="1"/>
+      <c r="X22" s="1"/>
+    </row>
+    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S23" s="1"/>
-      <c r="T23" s="3"/>
-      <c r="V23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="3"/>
       <c r="W23" s="1"/>
-    </row>
-    <row r="24" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="O24" s="2"/>
-      <c r="R24" s="1"/>
+      <c r="X23" s="1"/>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S24" s="1"/>
-      <c r="T24" s="3"/>
-      <c r="V24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="3"/>
       <c r="W24" s="1"/>
-    </row>
-    <row r="25" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="O25" s="2"/>
-      <c r="R25" s="1"/>
+      <c r="X24" s="1"/>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S25" s="1"/>
-      <c r="T25" s="3"/>
-      <c r="V25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="3"/>
       <c r="W25" s="1"/>
-    </row>
-    <row r="26" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="O26" s="2"/>
-      <c r="R26" s="1"/>
+      <c r="X25" s="1"/>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S26" s="1"/>
-      <c r="T26" s="3"/>
-      <c r="V26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="3"/>
       <c r="W26" s="1"/>
-    </row>
-    <row r="27" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R27" s="1"/>
+      <c r="X26" s="1"/>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="P27" s="2"/>
       <c r="S27" s="1"/>
-      <c r="T27" s="3"/>
-      <c r="V27" s="1"/>
+      <c r="T27" s="1"/>
+      <c r="U27" s="3"/>
       <c r="W27" s="1"/>
-    </row>
-    <row r="28" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R28" s="1"/>
+      <c r="X27" s="1"/>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="P28" s="2"/>
       <c r="S28" s="1"/>
-      <c r="T28" s="3"/>
-      <c r="V28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="3"/>
       <c r="W28" s="1"/>
-    </row>
-    <row r="29" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R29" s="1"/>
+      <c r="X28" s="1"/>
+    </row>
+    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="P29" s="2"/>
       <c r="S29" s="1"/>
-      <c r="T29" s="3"/>
-      <c r="V29" s="1"/>
+      <c r="T29" s="1"/>
+      <c r="U29" s="3"/>
       <c r="W29" s="1"/>
-    </row>
-    <row r="30" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R30" s="1"/>
+      <c r="X29" s="1"/>
+    </row>
+    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S30" s="1"/>
-      <c r="T30" s="3"/>
-      <c r="V30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="3"/>
       <c r="W30" s="1"/>
-    </row>
-    <row r="31" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R31" s="1"/>
+      <c r="X30" s="1"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S31" s="1"/>
-      <c r="T31" s="3"/>
-      <c r="V31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="3"/>
       <c r="W31" s="1"/>
-    </row>
-    <row r="32" spans="15:23" x14ac:dyDescent="0.2">
-      <c r="R32" s="1"/>
+      <c r="X31" s="1"/>
+    </row>
+    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="S32" s="1"/>
-      <c r="T32" s="3"/>
-      <c r="V32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="3"/>
       <c r="W32" s="1"/>
-    </row>
-    <row r="33" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="P33" s="2"/>
-      <c r="R33" s="1"/>
+      <c r="X32" s="1"/>
+    </row>
+    <row r="33" spans="6:24" x14ac:dyDescent="0.2">
       <c r="S33" s="1"/>
-      <c r="T33" s="3"/>
-      <c r="V33" s="1"/>
+      <c r="T33" s="1"/>
+      <c r="U33" s="3"/>
       <c r="W33" s="1"/>
-    </row>
-    <row r="34" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="R34" s="1"/>
+      <c r="X33" s="1"/>
+    </row>
+    <row r="34" spans="6:24" x14ac:dyDescent="0.2">
       <c r="S34" s="1"/>
-      <c r="T34" s="3"/>
-      <c r="V34" s="1"/>
+      <c r="T34" s="1"/>
+      <c r="U34" s="3"/>
       <c r="W34" s="1"/>
-    </row>
-    <row r="35" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="R35" s="1"/>
+      <c r="X34" s="1"/>
+    </row>
+    <row r="35" spans="6:24" x14ac:dyDescent="0.2">
       <c r="S35" s="1"/>
-      <c r="T35" s="3"/>
-      <c r="V35" s="1"/>
+      <c r="T35" s="1"/>
+      <c r="U35" s="3"/>
       <c r="W35" s="1"/>
-    </row>
-    <row r="36" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="R36" s="1"/>
-    </row>
-    <row r="37" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="R37" s="1"/>
-    </row>
-    <row r="38" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="K38" s="4"/>
-      <c r="L38" s="4"/>
-      <c r="R38" s="1"/>
-    </row>
-    <row r="39" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="R39" s="1"/>
+      <c r="X35" s="1"/>
+    </row>
+    <row r="36" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="Q36" s="2"/>
+      <c r="S36" s="1"/>
+      <c r="T36" s="1"/>
+      <c r="U36" s="3"/>
+      <c r="W36" s="1"/>
+      <c r="X36" s="1"/>
+    </row>
+    <row r="37" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="S37" s="1"/>
+      <c r="T37" s="1"/>
+      <c r="U37" s="3"/>
+      <c r="W37" s="1"/>
+      <c r="X37" s="1"/>
+    </row>
+    <row r="38" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="S38" s="1"/>
+      <c r="T38" s="1"/>
+      <c r="U38" s="3"/>
+      <c r="W38" s="1"/>
+      <c r="X38" s="1"/>
+    </row>
+    <row r="39" spans="6:24" x14ac:dyDescent="0.2">
       <c r="S39" s="1"/>
-      <c r="T39" s="3"/>
-      <c r="V39" s="1"/>
-      <c r="W39" s="1"/>
-    </row>
-    <row r="40" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="E40">
-        <v>1</v>
-      </c>
-      <c r="V40" s="1">
+    </row>
+    <row r="40" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="S40" s="1"/>
+    </row>
+    <row r="41" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="S41" s="1"/>
+    </row>
+    <row r="42" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="S42" s="1"/>
+      <c r="T42" s="1"/>
+      <c r="U42" s="3"/>
+      <c r="W42" s="1"/>
+      <c r="X42" s="1"/>
+    </row>
+    <row r="43" spans="6:24" x14ac:dyDescent="0.2">
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="W43" s="1">
         <v>2</v>
       </c>
-      <c r="W40" s="1"/>
-    </row>
-    <row r="48" spans="5:23" x14ac:dyDescent="0.2">
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-      <c r="P48" s="1"/>
-    </row>
-    <row r="56" spans="13:13" x14ac:dyDescent="0.2">
-      <c r="M56" s="5"/>
-    </row>
-    <row r="57" spans="13:13" x14ac:dyDescent="0.2">
-      <c r="M57" s="4"/>
+      <c r="X43" s="1"/>
+    </row>
+    <row r="51" spans="12:17" x14ac:dyDescent="0.2">
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+      <c r="Q51" s="1"/>
+    </row>
+    <row r="59" spans="12:17" x14ac:dyDescent="0.2">
+      <c r="N59" s="5"/>
+    </row>
+    <row r="60" spans="12:17" x14ac:dyDescent="0.2">
+      <c r="N60" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>